<commit_message>
Add status-color donut legends across all pages, H1/H2 RTM toggle, wire header stats to specific Excel cells (M65/U65/M66), fix TypeScript build errors
</commit_message>
<xml_diff>
--- a/files/Business Plan Final Ver 1.6.xlsx
+++ b/files/Business Plan Final Ver 1.6.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30305"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30306"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://techpayai-my.sharepoint.com/personal/shiv_kumar_techpay_ai/Documents/Documents/Office Related/Galaxy Target Letter/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5FD48F35-7E0E-48E7-A6B2-F0947E6DEDF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB407598-ABD6-4F1E-BDD0-6ADDBF6E94C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="599" firstSheet="4" activeTab="4" xr2:uid="{396E7889-4A15-A546-8860-B8AE67AFAEDB}"/>
   </bookViews>
@@ -3675,45 +3675,45 @@
     <xf numFmtId="171" fontId="18" fillId="0" borderId="1" xfId="11" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="17" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="19" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="6" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="43" fontId="19" fillId="5" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="6" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3726,6 +3726,12 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="10" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3738,33 +3744,27 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="7" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="2" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="3" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="4" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="7" xfId="13" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="5" xfId="13" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="6" xfId="13" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="7" xfId="13" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="5" xfId="13" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="6" xfId="13" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="2" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="3" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="4" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3804,6 +3804,15 @@
     <xf numFmtId="0" fontId="22" fillId="2" borderId="1" xfId="17" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3828,38 +3837,29 @@
     <xf numFmtId="0" fontId="20" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="7" xfId="14" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="14" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="14" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="7" xfId="14" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="14" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="14" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="12" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
@@ -4300,40 +4300,40 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:9">
-      <c r="B3" s="345" t="s">
+      <c r="B3" s="350" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="345"/>
-      <c r="D3" s="345"/>
-      <c r="E3" s="345"/>
-      <c r="F3" s="345"/>
-      <c r="G3" s="345"/>
-      <c r="H3" s="345"/>
-      <c r="I3" s="345"/>
+      <c r="C3" s="350"/>
+      <c r="D3" s="350"/>
+      <c r="E3" s="350"/>
+      <c r="F3" s="350"/>
+      <c r="G3" s="350"/>
+      <c r="H3" s="350"/>
+      <c r="I3" s="350"/>
     </row>
     <row r="4" spans="2:9">
-      <c r="B4" s="346" t="s">
+      <c r="B4" s="347" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="346" t="s">
+      <c r="C4" s="347" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="346" t="s">
+      <c r="D4" s="347" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="346"/>
-      <c r="F4" s="346" t="s">
+      <c r="E4" s="347"/>
+      <c r="F4" s="347" t="s">
         <v>4</v>
       </c>
-      <c r="G4" s="346"/>
-      <c r="H4" s="346" t="s">
+      <c r="G4" s="347"/>
+      <c r="H4" s="347" t="s">
         <v>5</v>
       </c>
-      <c r="I4" s="346"/>
+      <c r="I4" s="347"/>
     </row>
     <row r="5" spans="2:9">
-      <c r="B5" s="346"/>
-      <c r="C5" s="346"/>
+      <c r="B5" s="347"/>
+      <c r="C5" s="347"/>
       <c r="D5" s="101" t="s">
         <v>6</v>
       </c>
@@ -4618,40 +4618,40 @@
       </c>
     </row>
     <row r="16" spans="2:9">
-      <c r="B16" s="345" t="s">
+      <c r="B16" s="350" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="345"/>
-      <c r="D16" s="345"/>
-      <c r="E16" s="345"/>
-      <c r="F16" s="345"/>
-      <c r="G16" s="345"/>
-      <c r="H16" s="345"/>
-      <c r="I16" s="345"/>
+      <c r="C16" s="350"/>
+      <c r="D16" s="350"/>
+      <c r="E16" s="350"/>
+      <c r="F16" s="350"/>
+      <c r="G16" s="350"/>
+      <c r="H16" s="350"/>
+      <c r="I16" s="350"/>
     </row>
     <row r="17" spans="2:10">
-      <c r="B17" s="346" t="s">
+      <c r="B17" s="347" t="s">
         <v>1</v>
       </c>
-      <c r="C17" s="346" t="s">
+      <c r="C17" s="347" t="s">
         <v>2</v>
       </c>
-      <c r="D17" s="346" t="s">
+      <c r="D17" s="347" t="s">
         <v>3</v>
       </c>
-      <c r="E17" s="346"/>
-      <c r="F17" s="346" t="s">
+      <c r="E17" s="347"/>
+      <c r="F17" s="347" t="s">
         <v>4</v>
       </c>
-      <c r="G17" s="346"/>
-      <c r="H17" s="346" t="s">
+      <c r="G17" s="347"/>
+      <c r="H17" s="347" t="s">
         <v>5</v>
       </c>
-      <c r="I17" s="346"/>
+      <c r="I17" s="347"/>
     </row>
     <row r="18" spans="2:10">
-      <c r="B18" s="346"/>
-      <c r="C18" s="346"/>
+      <c r="B18" s="347"/>
+      <c r="C18" s="347"/>
       <c r="D18" s="101" t="s">
         <v>6</v>
       </c>
@@ -4934,40 +4934,40 @@
       </c>
     </row>
     <row r="29" spans="2:10">
-      <c r="B29" s="345" t="s">
+      <c r="B29" s="350" t="s">
         <v>17</v>
       </c>
-      <c r="C29" s="345"/>
-      <c r="D29" s="345"/>
-      <c r="E29" s="345"/>
-      <c r="F29" s="345"/>
-      <c r="G29" s="345"/>
-      <c r="H29" s="345"/>
-      <c r="I29" s="345"/>
+      <c r="C29" s="350"/>
+      <c r="D29" s="350"/>
+      <c r="E29" s="350"/>
+      <c r="F29" s="350"/>
+      <c r="G29" s="350"/>
+      <c r="H29" s="350"/>
+      <c r="I29" s="350"/>
     </row>
     <row r="30" spans="2:10">
-      <c r="B30" s="346" t="s">
+      <c r="B30" s="347" t="s">
         <v>1</v>
       </c>
-      <c r="C30" s="346" t="s">
+      <c r="C30" s="347" t="s">
         <v>2</v>
       </c>
-      <c r="D30" s="346" t="s">
+      <c r="D30" s="347" t="s">
         <v>3</v>
       </c>
-      <c r="E30" s="346"/>
-      <c r="F30" s="346" t="s">
+      <c r="E30" s="347"/>
+      <c r="F30" s="347" t="s">
         <v>4</v>
       </c>
-      <c r="G30" s="346"/>
-      <c r="H30" s="346" t="s">
+      <c r="G30" s="347"/>
+      <c r="H30" s="347" t="s">
         <v>5</v>
       </c>
-      <c r="I30" s="346"/>
+      <c r="I30" s="347"/>
     </row>
     <row r="31" spans="2:10">
-      <c r="B31" s="346"/>
-      <c r="C31" s="346"/>
+      <c r="B31" s="347"/>
+      <c r="C31" s="347"/>
       <c r="D31" s="101" t="s">
         <v>6</v>
       </c>
@@ -5255,40 +5255,40 @@
       <c r="N40" s="296"/>
     </row>
     <row r="42" spans="2:15" s="99" customFormat="1">
-      <c r="B42" s="347" t="s">
+      <c r="B42" s="348" t="s">
         <v>1</v>
       </c>
-      <c r="C42" s="347" t="s">
+      <c r="C42" s="348" t="s">
         <v>18</v>
       </c>
-      <c r="D42" s="349" t="s">
+      <c r="D42" s="345" t="s">
         <v>19</v>
       </c>
-      <c r="E42" s="350"/>
-      <c r="F42" s="349" t="s">
+      <c r="E42" s="346"/>
+      <c r="F42" s="345" t="s">
         <v>20</v>
       </c>
-      <c r="G42" s="350"/>
-      <c r="H42" s="349" t="s">
+      <c r="G42" s="346"/>
+      <c r="H42" s="345" t="s">
         <v>21</v>
       </c>
-      <c r="I42" s="350"/>
-      <c r="J42" s="349" t="s">
+      <c r="I42" s="346"/>
+      <c r="J42" s="345" t="s">
         <v>22</v>
       </c>
-      <c r="K42" s="350"/>
-      <c r="L42" s="349" t="s">
+      <c r="K42" s="346"/>
+      <c r="L42" s="345" t="s">
         <v>23</v>
       </c>
-      <c r="M42" s="350"/>
-      <c r="N42" s="349" t="s">
+      <c r="M42" s="346"/>
+      <c r="N42" s="345" t="s">
         <v>24</v>
       </c>
-      <c r="O42" s="350"/>
+      <c r="O42" s="346"/>
     </row>
     <row r="43" spans="2:15" s="99" customFormat="1">
-      <c r="B43" s="348"/>
-      <c r="C43" s="348"/>
+      <c r="B43" s="349"/>
+      <c r="C43" s="349"/>
       <c r="D43" s="101" t="s">
         <v>3</v>
       </c>
@@ -5845,17 +5845,6 @@
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="J42:K42"/>
-    <mergeCell ref="L42:M42"/>
-    <mergeCell ref="N42:O42"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="B42:B43"/>
-    <mergeCell ref="C42:C43"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="F42:G42"/>
-    <mergeCell ref="H42:I42"/>
     <mergeCell ref="B3:I3"/>
     <mergeCell ref="B16:I16"/>
     <mergeCell ref="B29:I29"/>
@@ -5871,6 +5860,17 @@
     <mergeCell ref="F17:G17"/>
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="C4:C5"/>
+    <mergeCell ref="B42:B43"/>
+    <mergeCell ref="C42:C43"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="F42:G42"/>
+    <mergeCell ref="H42:I42"/>
+    <mergeCell ref="J42:K42"/>
+    <mergeCell ref="L42:M42"/>
+    <mergeCell ref="N42:O42"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:I4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5915,26 +5915,26 @@
       </c>
     </row>
     <row r="6" spans="1:13">
-      <c r="A6" s="386" t="s">
+      <c r="A6" s="389" t="s">
         <v>36</v>
       </c>
-      <c r="B6" s="387"/>
-      <c r="C6" s="387"/>
-      <c r="D6" s="388"/>
+      <c r="B6" s="390"/>
+      <c r="C6" s="390"/>
+      <c r="D6" s="391"/>
       <c r="E6" s="114" t="s">
         <v>506</v>
       </c>
       <c r="F6" s="115" t="s">
         <v>507</v>
       </c>
-      <c r="G6" s="389" t="s">
+      <c r="G6" s="381" t="s">
         <v>212</v>
       </c>
-      <c r="H6" s="389"/>
-      <c r="I6" s="389" t="s">
+      <c r="H6" s="381"/>
+      <c r="I6" s="381" t="s">
         <v>213</v>
       </c>
-      <c r="J6" s="389"/>
+      <c r="J6" s="381"/>
     </row>
     <row r="7" spans="1:13" ht="26.45">
       <c r="A7" s="81" t="s">
@@ -5969,7 +5969,7 @@
       </c>
     </row>
     <row r="8" spans="1:13">
-      <c r="A8" s="390" t="s">
+      <c r="A8" s="382" t="s">
         <v>455</v>
       </c>
       <c r="B8" s="82" t="s">
@@ -6003,7 +6003,7 @@
       <c r="L8" s="291"/>
     </row>
     <row r="9" spans="1:13">
-      <c r="A9" s="390"/>
+      <c r="A9" s="382"/>
       <c r="B9" s="82" t="s">
         <v>216</v>
       </c>
@@ -6051,23 +6051,23 @@
     <row r="12" spans="1:13">
       <c r="A12" s="82"/>
       <c r="B12" s="116"/>
-      <c r="C12" s="389" t="s">
+      <c r="C12" s="381" t="s">
         <v>212</v>
       </c>
-      <c r="D12" s="389"/>
-      <c r="E12" s="389" t="s">
+      <c r="D12" s="381"/>
+      <c r="E12" s="381" t="s">
         <v>213</v>
       </c>
-      <c r="F12" s="389"/>
+      <c r="F12" s="381"/>
       <c r="G12" s="117"/>
-      <c r="H12" s="391" t="s">
+      <c r="H12" s="383" t="s">
         <v>212</v>
       </c>
-      <c r="I12" s="391"/>
-      <c r="J12" s="391" t="s">
+      <c r="I12" s="383"/>
+      <c r="J12" s="383" t="s">
         <v>213</v>
       </c>
-      <c r="K12" s="391"/>
+      <c r="K12" s="383"/>
       <c r="L12" s="317" t="s">
         <v>466</v>
       </c>
@@ -6272,9 +6272,9 @@
       <c r="L17" s="320"/>
     </row>
     <row r="19" spans="1:12">
-      <c r="A19" s="381"/>
-      <c r="B19" s="382"/>
-      <c r="C19" s="383"/>
+      <c r="A19" s="384"/>
+      <c r="B19" s="385"/>
+      <c r="C19" s="386"/>
     </row>
     <row r="20" spans="1:12">
       <c r="A20" s="81" t="s">
@@ -6412,10 +6412,10 @@
       <c r="E28" s="92"/>
     </row>
     <row r="29" spans="1:12">
-      <c r="B29" s="384" t="s">
+      <c r="B29" s="387" t="s">
         <v>515</v>
       </c>
-      <c r="C29" s="384"/>
+      <c r="C29" s="387"/>
       <c r="D29" s="93"/>
       <c r="E29" s="92"/>
     </row>
@@ -6500,10 +6500,10 @@
       </c>
     </row>
     <row r="40" spans="1:4">
-      <c r="B40" s="385" t="s">
+      <c r="B40" s="388" t="s">
         <v>516</v>
       </c>
-      <c r="C40" s="385"/>
+      <c r="C40" s="388"/>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="90" t="s">
@@ -6566,6 +6566,11 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="A6:D6"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="I6:J6"/>
     <mergeCell ref="A8:A9"/>
@@ -6573,11 +6578,6 @@
     <mergeCell ref="E12:F12"/>
     <mergeCell ref="H12:I12"/>
     <mergeCell ref="J12:K12"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="A6:D6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -6703,12 +6703,12 @@
       <c r="A12" s="127">
         <v>3</v>
       </c>
-      <c r="B12" s="395" t="s">
+      <c r="B12" s="396" t="s">
         <v>525</v>
       </c>
-      <c r="C12" s="395"/>
-      <c r="D12" s="395"/>
-      <c r="E12" s="395"/>
+      <c r="C12" s="396"/>
+      <c r="D12" s="396"/>
+      <c r="E12" s="396"/>
       <c r="F12" s="129"/>
       <c r="G12" s="129"/>
       <c r="H12" s="129"/>
@@ -6969,11 +6969,11 @@
       <c r="B42" s="119" t="s">
         <v>549</v>
       </c>
-      <c r="C42" s="399" t="s">
+      <c r="C42" s="398" t="s">
         <v>550</v>
       </c>
-      <c r="D42" s="399"/>
-      <c r="E42" s="399"/>
+      <c r="D42" s="398"/>
+      <c r="E42" s="398"/>
       <c r="F42" s="129"/>
       <c r="G42" s="129"/>
       <c r="H42" s="129"/>
@@ -6988,11 +6988,11 @@
       <c r="B43" s="120" t="s">
         <v>551</v>
       </c>
-      <c r="C43" s="394" t="s">
+      <c r="C43" s="392" t="s">
         <v>552</v>
       </c>
-      <c r="D43" s="394"/>
-      <c r="E43" s="394"/>
+      <c r="D43" s="392"/>
+      <c r="E43" s="392"/>
       <c r="F43" s="129"/>
       <c r="G43" s="129"/>
       <c r="H43" s="129"/>
@@ -7007,11 +7007,11 @@
       <c r="B44" s="120" t="s">
         <v>553</v>
       </c>
-      <c r="C44" s="394" t="s">
+      <c r="C44" s="392" t="s">
         <v>554</v>
       </c>
-      <c r="D44" s="394"/>
-      <c r="E44" s="394"/>
+      <c r="D44" s="392"/>
+      <c r="E44" s="392"/>
       <c r="F44" s="129"/>
       <c r="G44" s="129"/>
       <c r="H44" s="129"/>
@@ -7026,11 +7026,11 @@
       <c r="B45" s="120" t="s">
         <v>555</v>
       </c>
-      <c r="C45" s="394" t="s">
+      <c r="C45" s="392" t="s">
         <v>556</v>
       </c>
-      <c r="D45" s="394"/>
-      <c r="E45" s="394"/>
+      <c r="D45" s="392"/>
+      <c r="E45" s="392"/>
       <c r="F45" s="129"/>
       <c r="G45" s="129"/>
       <c r="H45" s="129"/>
@@ -7045,11 +7045,11 @@
       <c r="B46" s="120" t="s">
         <v>557</v>
       </c>
-      <c r="C46" s="394" t="s">
+      <c r="C46" s="392" t="s">
         <v>558</v>
       </c>
-      <c r="D46" s="394"/>
-      <c r="E46" s="394"/>
+      <c r="D46" s="392"/>
+      <c r="E46" s="392"/>
       <c r="F46" s="129"/>
       <c r="G46" s="129"/>
       <c r="H46" s="129"/>
@@ -7064,11 +7064,11 @@
       <c r="B47" s="120" t="s">
         <v>559</v>
       </c>
-      <c r="C47" s="394" t="s">
+      <c r="C47" s="392" t="s">
         <v>560</v>
       </c>
-      <c r="D47" s="394"/>
-      <c r="E47" s="394"/>
+      <c r="D47" s="392"/>
+      <c r="E47" s="392"/>
       <c r="F47" s="129"/>
       <c r="G47" s="129"/>
       <c r="H47" s="129"/>
@@ -7098,12 +7098,12 @@
       <c r="A49" s="127">
         <v>9</v>
       </c>
-      <c r="B49" s="392" t="s">
+      <c r="B49" s="397" t="s">
         <v>561</v>
       </c>
-      <c r="C49" s="392"/>
-      <c r="D49" s="392"/>
-      <c r="E49" s="392"/>
+      <c r="C49" s="397"/>
+      <c r="D49" s="397"/>
+      <c r="E49" s="397"/>
       <c r="F49" s="129"/>
       <c r="G49" s="129"/>
       <c r="H49" s="129"/>
@@ -7153,11 +7153,11 @@
       <c r="B52" s="120" t="s">
         <v>563</v>
       </c>
-      <c r="C52" s="394" t="s">
+      <c r="C52" s="392" t="s">
         <v>564</v>
       </c>
-      <c r="D52" s="394"/>
-      <c r="E52" s="394"/>
+      <c r="D52" s="392"/>
+      <c r="E52" s="392"/>
       <c r="F52" s="129"/>
       <c r="G52" s="129"/>
       <c r="H52" s="129"/>
@@ -7172,11 +7172,11 @@
       <c r="B53" s="120" t="s">
         <v>565</v>
       </c>
-      <c r="C53" s="394" t="s">
+      <c r="C53" s="392" t="s">
         <v>566</v>
       </c>
-      <c r="D53" s="394"/>
-      <c r="E53" s="394"/>
+      <c r="D53" s="392"/>
+      <c r="E53" s="392"/>
       <c r="F53" s="129"/>
       <c r="G53" s="129"/>
       <c r="H53" s="129"/>
@@ -7191,11 +7191,11 @@
       <c r="B54" s="120" t="s">
         <v>567</v>
       </c>
-      <c r="C54" s="394" t="s">
+      <c r="C54" s="392" t="s">
         <v>568</v>
       </c>
-      <c r="D54" s="394"/>
-      <c r="E54" s="394"/>
+      <c r="D54" s="392"/>
+      <c r="E54" s="392"/>
       <c r="F54" s="129"/>
       <c r="G54" s="129"/>
       <c r="H54" s="129"/>
@@ -7210,11 +7210,11 @@
       <c r="B55" s="120" t="s">
         <v>569</v>
       </c>
-      <c r="C55" s="394" t="s">
+      <c r="C55" s="392" t="s">
         <v>570</v>
       </c>
-      <c r="D55" s="394"/>
-      <c r="E55" s="394"/>
+      <c r="D55" s="392"/>
+      <c r="E55" s="392"/>
       <c r="F55" s="129"/>
       <c r="G55" s="129"/>
       <c r="H55" s="129"/>
@@ -7229,11 +7229,11 @@
       <c r="B56" s="120" t="s">
         <v>571</v>
       </c>
-      <c r="C56" s="394" t="s">
+      <c r="C56" s="392" t="s">
         <v>572</v>
       </c>
-      <c r="D56" s="394"/>
-      <c r="E56" s="394"/>
+      <c r="D56" s="392"/>
+      <c r="E56" s="392"/>
       <c r="F56" s="129"/>
       <c r="G56" s="129"/>
       <c r="H56" s="129"/>
@@ -7248,11 +7248,11 @@
       <c r="B57" s="120" t="s">
         <v>573</v>
       </c>
-      <c r="C57" s="394" t="s">
+      <c r="C57" s="392" t="s">
         <v>574</v>
       </c>
-      <c r="D57" s="394"/>
-      <c r="E57" s="394"/>
+      <c r="D57" s="392"/>
+      <c r="E57" s="392"/>
       <c r="F57" s="129"/>
       <c r="G57" s="129"/>
       <c r="H57" s="129"/>
@@ -7282,12 +7282,12 @@
       <c r="A59" s="127">
         <v>11</v>
       </c>
-      <c r="B59" s="395" t="s">
+      <c r="B59" s="396" t="s">
         <v>575</v>
       </c>
-      <c r="C59" s="395"/>
-      <c r="D59" s="395"/>
-      <c r="E59" s="395"/>
+      <c r="C59" s="396"/>
+      <c r="D59" s="396"/>
+      <c r="E59" s="396"/>
       <c r="F59" s="129"/>
       <c r="G59" s="129"/>
       <c r="H59" s="129"/>
@@ -7365,7 +7365,7 @@
       <c r="D63" s="123" t="s">
         <v>583</v>
       </c>
-      <c r="E63" s="396" t="s">
+      <c r="E63" s="393" t="s">
         <v>584</v>
       </c>
       <c r="F63" s="129"/>
@@ -7387,7 +7387,7 @@
       <c r="D64" s="124" t="s">
         <v>587</v>
       </c>
-      <c r="E64" s="397"/>
+      <c r="E64" s="394"/>
       <c r="F64" s="129"/>
       <c r="G64" s="129"/>
       <c r="H64" s="129"/>
@@ -7407,7 +7407,7 @@
       <c r="D65" s="124" t="s">
         <v>589</v>
       </c>
-      <c r="E65" s="398"/>
+      <c r="E65" s="395"/>
       <c r="F65" s="129"/>
       <c r="G65" s="129"/>
       <c r="H65" s="129"/>
@@ -7454,12 +7454,12 @@
       <c r="A71" s="127">
         <v>15</v>
       </c>
-      <c r="B71" s="393" t="s">
+      <c r="B71" s="399" t="s">
         <v>592</v>
       </c>
-      <c r="C71" s="393"/>
-      <c r="D71" s="393"/>
-      <c r="E71" s="393"/>
+      <c r="C71" s="399"/>
+      <c r="D71" s="399"/>
+      <c r="E71" s="399"/>
       <c r="F71" s="143"/>
       <c r="G71" s="143"/>
       <c r="H71" s="143"/>
@@ -7489,12 +7489,12 @@
       <c r="A73" s="127">
         <v>16</v>
       </c>
-      <c r="B73" s="395" t="s">
+      <c r="B73" s="396" t="s">
         <v>593</v>
       </c>
-      <c r="C73" s="395"/>
-      <c r="D73" s="395"/>
-      <c r="E73" s="395"/>
+      <c r="C73" s="396"/>
+      <c r="D73" s="396"/>
+      <c r="E73" s="396"/>
       <c r="F73" s="129"/>
       <c r="G73" s="129"/>
       <c r="H73" s="129"/>
@@ -7524,12 +7524,12 @@
       <c r="A75" s="127">
         <v>17</v>
       </c>
-      <c r="B75" s="392" t="s">
+      <c r="B75" s="397" t="s">
         <v>594</v>
       </c>
-      <c r="C75" s="392"/>
-      <c r="D75" s="392"/>
-      <c r="E75" s="392"/>
+      <c r="C75" s="397"/>
+      <c r="D75" s="397"/>
+      <c r="E75" s="397"/>
       <c r="F75" s="129"/>
       <c r="G75" s="129"/>
       <c r="H75" s="129"/>
@@ -7542,6 +7542,13 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="B75:E75"/>
+    <mergeCell ref="B71:E71"/>
+    <mergeCell ref="C55:E55"/>
+    <mergeCell ref="C56:E56"/>
+    <mergeCell ref="C57:E57"/>
+    <mergeCell ref="B59:E59"/>
+    <mergeCell ref="B73:E73"/>
     <mergeCell ref="C46:E46"/>
     <mergeCell ref="C47:E47"/>
     <mergeCell ref="E63:E65"/>
@@ -7554,13 +7561,6 @@
     <mergeCell ref="C43:E43"/>
     <mergeCell ref="C44:E44"/>
     <mergeCell ref="C45:E45"/>
-    <mergeCell ref="B75:E75"/>
-    <mergeCell ref="B71:E71"/>
-    <mergeCell ref="C55:E55"/>
-    <mergeCell ref="C56:E56"/>
-    <mergeCell ref="C57:E57"/>
-    <mergeCell ref="B59:E59"/>
-    <mergeCell ref="B73:E73"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9488,50 +9488,50 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:13" ht="15.6">
-      <c r="A2" s="356" t="s">
+      <c r="A2" s="358" t="s">
         <v>87</v>
       </c>
-      <c r="B2" s="356"/>
-      <c r="C2" s="356"/>
-      <c r="D2" s="356"/>
+      <c r="B2" s="358"/>
+      <c r="C2" s="358"/>
+      <c r="D2" s="358"/>
     </row>
     <row r="3" spans="1:13">
-      <c r="A3" s="357" t="s">
+      <c r="A3" s="359" t="s">
         <v>88</v>
       </c>
-      <c r="B3" s="357"/>
-      <c r="C3" s="357"/>
+      <c r="B3" s="359"/>
+      <c r="C3" s="359"/>
       <c r="D3" s="31" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:13">
-      <c r="A4" s="358" t="s">
+      <c r="A4" s="360" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="358"/>
-      <c r="C4" s="358"/>
+      <c r="B4" s="360"/>
+      <c r="C4" s="360"/>
       <c r="D4" s="32">
         <v>310</v>
       </c>
     </row>
     <row r="5" spans="1:13">
-      <c r="A5" s="358" t="s">
+      <c r="A5" s="360" t="s">
         <v>40</v>
       </c>
-      <c r="B5" s="358"/>
-      <c r="C5" s="358"/>
+      <c r="B5" s="360"/>
+      <c r="C5" s="360"/>
       <c r="D5" s="33">
         <f>D4*8%</f>
         <v>24.8</v>
       </c>
     </row>
     <row r="6" spans="1:13">
-      <c r="A6" s="358" t="s">
+      <c r="A6" s="360" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="358"/>
-      <c r="C6" s="358"/>
+      <c r="B6" s="360"/>
+      <c r="C6" s="360"/>
       <c r="D6" s="33">
         <f>D4*2%</f>
         <v>6.2</v>
@@ -9539,11 +9539,11 @@
     </row>
     <row r="8" spans="1:13">
       <c r="B8" s="34"/>
-      <c r="K8" s="355" t="s">
+      <c r="K8" s="357" t="s">
         <v>90</v>
       </c>
-      <c r="L8" s="355"/>
-      <c r="M8" s="355"/>
+      <c r="L8" s="357"/>
+      <c r="M8" s="357"/>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="36" t="s">
@@ -10684,11 +10684,11 @@
       </c>
     </row>
     <row r="35" spans="1:13" s="34" customFormat="1">
-      <c r="A35" s="359" t="s">
+      <c r="A35" s="355" t="s">
         <v>15</v>
       </c>
-      <c r="B35" s="359"/>
-      <c r="C35" s="359"/>
+      <c r="B35" s="355"/>
+      <c r="C35" s="355"/>
       <c r="D35" s="42">
         <f>SUM(D10:D34)</f>
         <v>310</v>
@@ -10713,11 +10713,11 @@
       <c r="J35" s="43"/>
     </row>
     <row r="38" spans="1:13">
-      <c r="A38" s="360" t="s">
+      <c r="A38" s="356" t="s">
         <v>193</v>
       </c>
-      <c r="B38" s="360"/>
-      <c r="C38" s="360"/>
+      <c r="B38" s="356"/>
+      <c r="C38" s="356"/>
       <c r="D38" s="31" t="s">
         <v>93</v>
       </c>
@@ -10800,11 +10800,11 @@
       <c r="E45" s="44"/>
     </row>
     <row r="46" spans="1:13">
-      <c r="A46" s="359" t="s">
+      <c r="A46" s="355" t="s">
         <v>15</v>
       </c>
-      <c r="B46" s="359"/>
-      <c r="C46" s="359"/>
+      <c r="B46" s="355"/>
+      <c r="C46" s="355"/>
       <c r="D46" s="42">
         <f>SUM(D39:D45)</f>
         <v>300</v>
@@ -10812,6 +10812,12 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="K8:M8"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A6:C6"/>
     <mergeCell ref="A43:C43"/>
     <mergeCell ref="A44:C44"/>
     <mergeCell ref="A45:C45"/>
@@ -10822,12 +10828,6 @@
     <mergeCell ref="A40:C40"/>
     <mergeCell ref="A41:C41"/>
     <mergeCell ref="A42:C42"/>
-    <mergeCell ref="K8:M8"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A6:C6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -11068,18 +11068,18 @@
       <c r="D4" s="50"/>
     </row>
     <row r="6" spans="1:12">
-      <c r="C6" s="338"/>
-      <c r="D6" s="338"/>
-      <c r="E6" s="338"/>
+      <c r="C6" s="343"/>
+      <c r="D6" s="343"/>
+      <c r="E6" s="343"/>
       <c r="G6" s="107"/>
-      <c r="H6" s="339" t="s">
+      <c r="H6" s="344" t="s">
         <v>212</v>
       </c>
-      <c r="I6" s="339"/>
-      <c r="J6" s="339" t="s">
+      <c r="I6" s="344"/>
+      <c r="J6" s="344" t="s">
         <v>213</v>
       </c>
-      <c r="K6" s="339"/>
+      <c r="K6" s="344"/>
     </row>
     <row r="7" spans="1:12">
       <c r="C7" s="84" t="s">
@@ -11166,19 +11166,19 @@
       </c>
     </row>
     <row r="11" spans="1:12">
-      <c r="C11" s="338"/>
-      <c r="D11" s="338"/>
-      <c r="E11" s="338"/>
-      <c r="F11" s="338"/>
+      <c r="C11" s="343"/>
+      <c r="D11" s="343"/>
+      <c r="E11" s="343"/>
+      <c r="F11" s="343"/>
       <c r="G11" s="105"/>
-      <c r="H11" s="339" t="s">
+      <c r="H11" s="344" t="s">
         <v>212</v>
       </c>
-      <c r="I11" s="339"/>
-      <c r="J11" s="339" t="s">
+      <c r="I11" s="344"/>
+      <c r="J11" s="344" t="s">
         <v>213</v>
       </c>
-      <c r="K11" s="339"/>
+      <c r="K11" s="344"/>
       <c r="L11" s="275" t="s">
         <v>217</v>
       </c>
@@ -11223,7 +11223,7 @@
       <c r="B13" s="49" t="s">
         <v>221</v>
       </c>
-      <c r="C13" s="340" t="s">
+      <c r="C13" s="338" t="s">
         <v>222</v>
       </c>
       <c r="D13" s="54"/>
@@ -11249,7 +11249,7 @@
       <c r="B14" s="49" t="s">
         <v>221</v>
       </c>
-      <c r="C14" s="340"/>
+      <c r="C14" s="338"/>
       <c r="D14" s="54" t="s">
         <v>224</v>
       </c>
@@ -11275,7 +11275,7 @@
       <c r="B15" s="49" t="s">
         <v>221</v>
       </c>
-      <c r="C15" s="340"/>
+      <c r="C15" s="338"/>
       <c r="D15" s="54" t="s">
         <v>225</v>
       </c>
@@ -11296,7 +11296,7 @@
       <c r="B16" s="49" t="s">
         <v>221</v>
       </c>
-      <c r="C16" s="340"/>
+      <c r="C16" s="338"/>
       <c r="D16" s="54" t="s">
         <v>227</v>
       </c>
@@ -11317,7 +11317,7 @@
       <c r="B17" s="49" t="s">
         <v>221</v>
       </c>
-      <c r="C17" s="340"/>
+      <c r="C17" s="338"/>
       <c r="D17" s="54" t="s">
         <v>228</v>
       </c>
@@ -11338,7 +11338,7 @@
       <c r="B18" s="49" t="s">
         <v>221</v>
       </c>
-      <c r="C18" s="340"/>
+      <c r="C18" s="338"/>
       <c r="D18" s="54" t="s">
         <v>229</v>
       </c>
@@ -11364,7 +11364,7 @@
       <c r="B19" s="49" t="s">
         <v>221</v>
       </c>
-      <c r="C19" s="340"/>
+      <c r="C19" s="338"/>
       <c r="D19" s="54" t="s">
         <v>230</v>
       </c>
@@ -11385,7 +11385,7 @@
       <c r="B20" s="49" t="s">
         <v>221</v>
       </c>
-      <c r="C20" s="340"/>
+      <c r="C20" s="338"/>
       <c r="D20" s="54" t="s">
         <v>231</v>
       </c>
@@ -11411,7 +11411,7 @@
       <c r="B21" s="49" t="s">
         <v>221</v>
       </c>
-      <c r="C21" s="340"/>
+      <c r="C21" s="338"/>
       <c r="D21" s="54" t="s">
         <v>232</v>
       </c>
@@ -11432,7 +11432,7 @@
       <c r="B22" s="49" t="s">
         <v>221</v>
       </c>
-      <c r="C22" s="340"/>
+      <c r="C22" s="338"/>
       <c r="D22" s="54" t="s">
         <v>233</v>
       </c>
@@ -11561,7 +11561,7 @@
       <c r="B26" s="49" t="s">
         <v>221</v>
       </c>
-      <c r="C26" s="340" t="s">
+      <c r="C26" s="338" t="s">
         <v>238</v>
       </c>
       <c r="E26" s="48" t="s">
@@ -11586,7 +11586,7 @@
       <c r="B27" s="49" t="s">
         <v>221</v>
       </c>
-      <c r="C27" s="340"/>
+      <c r="C27" s="338"/>
       <c r="D27" s="53" t="s">
         <v>239</v>
       </c>
@@ -11611,7 +11611,7 @@
       <c r="B28" s="49" t="s">
         <v>221</v>
       </c>
-      <c r="C28" s="340"/>
+      <c r="C28" s="338"/>
       <c r="D28" s="53" t="s">
         <v>240</v>
       </c>
@@ -11636,7 +11636,7 @@
       <c r="B29" s="49" t="s">
         <v>221</v>
       </c>
-      <c r="C29" s="340"/>
+      <c r="C29" s="338"/>
       <c r="D29" s="53" t="s">
         <v>241</v>
       </c>
@@ -11661,7 +11661,7 @@
       <c r="B30" s="49" t="s">
         <v>221</v>
       </c>
-      <c r="C30" s="340"/>
+      <c r="C30" s="338"/>
       <c r="D30" s="53" t="s">
         <v>242</v>
       </c>
@@ -11686,7 +11686,7 @@
       <c r="B31" s="49" t="s">
         <v>221</v>
       </c>
-      <c r="C31" s="340"/>
+      <c r="C31" s="338"/>
       <c r="D31" s="53" t="s">
         <v>243</v>
       </c>
@@ -11855,7 +11855,7 @@
       <c r="B36" s="49" t="s">
         <v>245</v>
       </c>
-      <c r="C36" s="342" t="s">
+      <c r="C36" s="340" t="s">
         <v>249</v>
       </c>
       <c r="D36" s="54"/>
@@ -11881,7 +11881,7 @@
       <c r="B37" s="49" t="s">
         <v>245</v>
       </c>
-      <c r="C37" s="343"/>
+      <c r="C37" s="341"/>
       <c r="D37" s="54" t="s">
         <v>250</v>
       </c>
@@ -11904,7 +11904,7 @@
       <c r="B38" s="49" t="s">
         <v>245</v>
       </c>
-      <c r="C38" s="343"/>
+      <c r="C38" s="341"/>
       <c r="D38" s="54" t="s">
         <v>251</v>
       </c>
@@ -11927,7 +11927,7 @@
       <c r="B39" s="49" t="s">
         <v>245</v>
       </c>
-      <c r="C39" s="343"/>
+      <c r="C39" s="341"/>
       <c r="D39" s="54" t="s">
         <v>252</v>
       </c>
@@ -11950,7 +11950,7 @@
       <c r="B40" s="49" t="s">
         <v>245</v>
       </c>
-      <c r="C40" s="343"/>
+      <c r="C40" s="341"/>
       <c r="D40" s="54" t="s">
         <v>253</v>
       </c>
@@ -11973,7 +11973,7 @@
       <c r="B41" s="49" t="s">
         <v>245</v>
       </c>
-      <c r="C41" s="344"/>
+      <c r="C41" s="342"/>
       <c r="D41" s="54" t="s">
         <v>254</v>
       </c>
@@ -12030,7 +12030,7 @@
       <c r="B43" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C43" s="342" t="s">
+      <c r="C43" s="340" t="s">
         <v>257</v>
       </c>
       <c r="D43" s="53" t="s">
@@ -12066,7 +12066,7 @@
       <c r="B44" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C44" s="344"/>
+      <c r="C44" s="342"/>
       <c r="D44" s="53" t="s">
         <v>258</v>
       </c>
@@ -12094,7 +12094,7 @@
       <c r="B45" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C45" s="342" t="s">
+      <c r="C45" s="340" t="s">
         <v>259</v>
       </c>
       <c r="D45" s="53" t="s">
@@ -12130,7 +12130,7 @@
       <c r="B46" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C46" s="343"/>
+      <c r="C46" s="341"/>
       <c r="D46" s="55" t="s">
         <v>260</v>
       </c>
@@ -12158,7 +12158,7 @@
       <c r="B47" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C47" s="343"/>
+      <c r="C47" s="341"/>
       <c r="D47" s="55" t="s">
         <v>261</v>
       </c>
@@ -12177,7 +12177,7 @@
       <c r="B48" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C48" s="343"/>
+      <c r="C48" s="341"/>
       <c r="D48" s="279" t="s">
         <v>262</v>
       </c>
@@ -12197,7 +12197,7 @@
       <c r="B49" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C49" s="343"/>
+      <c r="C49" s="341"/>
       <c r="D49" s="279" t="s">
         <v>264</v>
       </c>
@@ -12217,7 +12217,7 @@
       <c r="B50" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C50" s="343"/>
+      <c r="C50" s="341"/>
       <c r="D50" s="279" t="s">
         <v>265</v>
       </c>
@@ -12237,7 +12237,7 @@
       <c r="B51" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C51" s="343"/>
+      <c r="C51" s="341"/>
       <c r="D51" s="279" t="s">
         <v>266</v>
       </c>
@@ -12257,7 +12257,7 @@
       <c r="B52" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C52" s="343"/>
+      <c r="C52" s="341"/>
       <c r="D52" s="279" t="s">
         <v>267</v>
       </c>
@@ -12277,7 +12277,7 @@
       <c r="B53" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C53" s="343"/>
+      <c r="C53" s="341"/>
       <c r="D53" s="279" t="s">
         <v>268</v>
       </c>
@@ -12297,7 +12297,7 @@
       <c r="B54" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C54" s="343"/>
+      <c r="C54" s="341"/>
       <c r="D54" s="279" t="s">
         <v>269</v>
       </c>
@@ -12317,7 +12317,7 @@
       <c r="B55" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C55" s="343"/>
+      <c r="C55" s="341"/>
       <c r="D55" s="279" t="s">
         <v>270</v>
       </c>
@@ -12337,7 +12337,7 @@
       <c r="B56" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C56" s="343"/>
+      <c r="C56" s="341"/>
       <c r="D56" s="279" t="s">
         <v>271</v>
       </c>
@@ -12357,7 +12357,7 @@
       <c r="B57" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C57" s="343"/>
+      <c r="C57" s="341"/>
       <c r="D57" s="279" t="s">
         <v>272</v>
       </c>
@@ -12377,7 +12377,7 @@
       <c r="B58" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C58" s="343"/>
+      <c r="C58" s="341"/>
       <c r="D58" s="279" t="s">
         <v>273</v>
       </c>
@@ -12397,7 +12397,7 @@
       <c r="B59" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C59" s="343"/>
+      <c r="C59" s="341"/>
       <c r="D59" s="279" t="s">
         <v>274</v>
       </c>
@@ -12417,7 +12417,7 @@
       <c r="B60" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C60" s="343"/>
+      <c r="C60" s="341"/>
       <c r="D60" s="279" t="s">
         <v>275</v>
       </c>
@@ -12437,7 +12437,7 @@
       <c r="B61" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C61" s="343"/>
+      <c r="C61" s="341"/>
       <c r="D61" s="279" t="s">
         <v>276</v>
       </c>
@@ -12457,7 +12457,7 @@
       <c r="B62" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C62" s="343"/>
+      <c r="C62" s="341"/>
       <c r="D62" s="279" t="s">
         <v>277</v>
       </c>
@@ -12477,7 +12477,7 @@
       <c r="B63" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C63" s="343"/>
+      <c r="C63" s="341"/>
       <c r="D63" s="279" t="s">
         <v>278</v>
       </c>
@@ -12497,7 +12497,7 @@
       <c r="B64" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C64" s="344"/>
+      <c r="C64" s="342"/>
       <c r="D64" s="279" t="s">
         <v>279</v>
       </c>
@@ -12550,7 +12550,7 @@
       <c r="B66" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C66" s="342" t="s">
+      <c r="C66" s="340" t="s">
         <v>280</v>
       </c>
       <c r="D66" s="313" t="s">
@@ -12577,7 +12577,7 @@
       <c r="B67" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C67" s="343"/>
+      <c r="C67" s="341"/>
       <c r="D67" s="313" t="s">
         <v>282</v>
       </c>
@@ -12597,7 +12597,7 @@
       <c r="B68" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C68" s="343"/>
+      <c r="C68" s="341"/>
       <c r="D68" s="313" t="s">
         <v>284</v>
       </c>
@@ -12617,7 +12617,7 @@
       <c r="B69" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C69" s="343"/>
+      <c r="C69" s="341"/>
       <c r="D69" s="313" t="s">
         <v>285</v>
       </c>
@@ -12637,7 +12637,7 @@
       <c r="B70" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C70" s="343"/>
+      <c r="C70" s="341"/>
       <c r="D70" s="313" t="s">
         <v>286</v>
       </c>
@@ -12657,7 +12657,7 @@
       <c r="B71" s="49" t="s">
         <v>256</v>
       </c>
-      <c r="C71" s="344"/>
+      <c r="C71" s="342"/>
       <c r="D71" s="313" t="s">
         <v>287</v>
       </c>
@@ -12702,7 +12702,7 @@
       <c r="B73" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C73" s="342" t="s">
+      <c r="C73" s="340" t="s">
         <v>290</v>
       </c>
       <c r="D73" s="53" t="s">
@@ -12723,7 +12723,7 @@
       <c r="B74" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C74" s="343"/>
+      <c r="C74" s="341"/>
       <c r="D74" s="53" t="s">
         <v>292</v>
       </c>
@@ -12746,7 +12746,7 @@
       <c r="B75" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C75" s="343"/>
+      <c r="C75" s="341"/>
       <c r="D75" s="53" t="s">
         <v>293</v>
       </c>
@@ -12765,7 +12765,7 @@
       <c r="B76" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C76" s="343"/>
+      <c r="C76" s="341"/>
       <c r="D76" s="53" t="s">
         <v>294</v>
       </c>
@@ -12784,7 +12784,7 @@
       <c r="B77" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C77" s="343"/>
+      <c r="C77" s="341"/>
       <c r="D77" s="53" t="s">
         <v>295</v>
       </c>
@@ -12807,7 +12807,7 @@
       <c r="B78" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C78" s="343"/>
+      <c r="C78" s="341"/>
       <c r="D78" s="53" t="s">
         <v>296</v>
       </c>
@@ -12830,7 +12830,7 @@
       <c r="B79" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C79" s="343"/>
+      <c r="C79" s="341"/>
       <c r="D79" s="53" t="s">
         <v>297</v>
       </c>
@@ -12853,7 +12853,7 @@
       <c r="B80" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C80" s="343"/>
+      <c r="C80" s="341"/>
       <c r="D80" s="53" t="s">
         <v>298</v>
       </c>
@@ -12876,7 +12876,7 @@
       <c r="B81" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C81" s="343"/>
+      <c r="C81" s="341"/>
       <c r="D81" s="53" t="s">
         <v>299</v>
       </c>
@@ -12901,7 +12901,7 @@
       <c r="B82" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C82" s="343"/>
+      <c r="C82" s="341"/>
       <c r="D82" s="53" t="s">
         <v>300</v>
       </c>
@@ -12924,7 +12924,7 @@
       <c r="B83" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C83" s="343"/>
+      <c r="C83" s="341"/>
       <c r="D83" s="53" t="s">
         <v>301</v>
       </c>
@@ -12949,7 +12949,7 @@
       <c r="B84" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C84" s="343"/>
+      <c r="C84" s="341"/>
       <c r="D84" s="53" t="s">
         <v>302</v>
       </c>
@@ -12974,7 +12974,7 @@
       <c r="B85" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C85" s="343"/>
+      <c r="C85" s="341"/>
       <c r="D85" s="309" t="s">
         <v>303</v>
       </c>
@@ -12993,7 +12993,7 @@
       <c r="B86" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C86" s="343"/>
+      <c r="C86" s="341"/>
       <c r="D86" s="309" t="s">
         <v>304</v>
       </c>
@@ -13012,7 +13012,7 @@
       <c r="B87" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C87" s="343"/>
+      <c r="C87" s="341"/>
       <c r="D87" s="309" t="s">
         <v>305</v>
       </c>
@@ -13031,7 +13031,7 @@
       <c r="B88" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C88" s="343"/>
+      <c r="C88" s="341"/>
       <c r="D88" s="309" t="s">
         <v>306</v>
       </c>
@@ -13050,7 +13050,7 @@
       <c r="B89" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C89" s="343"/>
+      <c r="C89" s="341"/>
       <c r="D89" s="309" t="s">
         <v>307</v>
       </c>
@@ -13069,7 +13069,7 @@
       <c r="B90" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C90" s="343"/>
+      <c r="C90" s="341"/>
       <c r="D90" s="309" t="s">
         <v>308</v>
       </c>
@@ -13088,7 +13088,7 @@
       <c r="B91" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C91" s="343"/>
+      <c r="C91" s="341"/>
       <c r="D91" s="309" t="s">
         <v>309</v>
       </c>
@@ -13105,7 +13105,7 @@
       <c r="B92" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C92" s="343"/>
+      <c r="C92" s="341"/>
       <c r="D92" s="309" t="s">
         <v>310</v>
       </c>
@@ -13124,7 +13124,7 @@
       <c r="B93" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C93" s="343"/>
+      <c r="C93" s="341"/>
       <c r="D93" s="309" t="s">
         <v>311</v>
       </c>
@@ -13143,7 +13143,7 @@
       <c r="B94" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C94" s="344"/>
+      <c r="C94" s="342"/>
       <c r="D94" s="309" t="s">
         <v>312</v>
       </c>
@@ -13185,7 +13185,7 @@
       <c r="B96" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C96" s="340" t="s">
+      <c r="C96" s="338" t="s">
         <v>314</v>
       </c>
       <c r="D96" s="53" t="s">
@@ -13212,7 +13212,7 @@
       <c r="B97" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C97" s="340"/>
+      <c r="C97" s="338"/>
       <c r="D97" s="53" t="s">
         <v>316</v>
       </c>
@@ -13237,7 +13237,7 @@
       <c r="B98" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C98" s="340"/>
+      <c r="C98" s="338"/>
       <c r="D98" s="53" t="s">
         <v>317</v>
       </c>
@@ -13262,7 +13262,7 @@
       <c r="B99" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C99" s="340"/>
+      <c r="C99" s="338"/>
       <c r="D99" s="53" t="s">
         <v>318</v>
       </c>
@@ -13287,7 +13287,7 @@
       <c r="B100" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C100" s="340"/>
+      <c r="C100" s="338"/>
       <c r="D100" s="53" t="s">
         <v>319</v>
       </c>
@@ -13306,7 +13306,7 @@
       <c r="B101" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C101" s="340"/>
+      <c r="C101" s="338"/>
       <c r="D101" s="53" t="s">
         <v>320</v>
       </c>
@@ -13329,7 +13329,7 @@
       <c r="B102" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C102" s="340"/>
+      <c r="C102" s="338"/>
       <c r="D102" s="53" t="s">
         <v>321</v>
       </c>
@@ -13350,7 +13350,7 @@
       <c r="B103" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C103" s="340"/>
+      <c r="C103" s="338"/>
       <c r="D103" s="53" t="s">
         <v>322</v>
       </c>
@@ -13367,7 +13367,7 @@
       <c r="B104" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C104" s="340"/>
+      <c r="C104" s="338"/>
       <c r="D104" s="53" t="s">
         <v>323</v>
       </c>
@@ -13386,7 +13386,7 @@
       <c r="B105" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C105" s="340"/>
+      <c r="C105" s="338"/>
       <c r="D105" s="53" t="s">
         <v>324</v>
       </c>
@@ -13409,7 +13409,7 @@
       <c r="B106" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C106" s="340"/>
+      <c r="C106" s="338"/>
       <c r="D106" s="53" t="s">
         <v>325</v>
       </c>
@@ -13434,7 +13434,7 @@
       <c r="B107" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C107" s="340"/>
+      <c r="C107" s="338"/>
       <c r="D107" s="53" t="s">
         <v>326</v>
       </c>
@@ -13457,7 +13457,7 @@
       <c r="B108" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C108" s="340"/>
+      <c r="C108" s="338"/>
       <c r="D108" s="53" t="s">
         <v>327</v>
       </c>
@@ -13480,7 +13480,7 @@
       <c r="B109" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C109" s="340"/>
+      <c r="C109" s="338"/>
       <c r="D109" s="53" t="s">
         <v>328</v>
       </c>
@@ -13503,7 +13503,7 @@
       <c r="B110" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="C110" s="340"/>
+      <c r="C110" s="338"/>
       <c r="D110" s="53" t="s">
         <v>329</v>
       </c>
@@ -13528,7 +13528,7 @@
       <c r="B111" s="49" t="s">
         <v>330</v>
       </c>
-      <c r="C111" s="340" t="s">
+      <c r="C111" s="338" t="s">
         <v>331</v>
       </c>
       <c r="D111" s="53" t="s">
@@ -13564,7 +13564,7 @@
       <c r="B112" s="49" t="s">
         <v>330</v>
       </c>
-      <c r="C112" s="340"/>
+      <c r="C112" s="338"/>
       <c r="D112" s="53" t="s">
         <v>333</v>
       </c>
@@ -13583,7 +13583,7 @@
       <c r="B113" s="49" t="s">
         <v>330</v>
       </c>
-      <c r="C113" s="340"/>
+      <c r="C113" s="338"/>
       <c r="D113" s="53" t="s">
         <v>334</v>
       </c>
@@ -13602,7 +13602,7 @@
       <c r="B114" s="49" t="s">
         <v>330</v>
       </c>
-      <c r="C114" s="340"/>
+      <c r="C114" s="338"/>
       <c r="D114" s="53" t="s">
         <v>335</v>
       </c>
@@ -13621,7 +13621,7 @@
       <c r="B115" s="49" t="s">
         <v>330</v>
       </c>
-      <c r="C115" s="340"/>
+      <c r="C115" s="338"/>
       <c r="D115" s="53" t="s">
         <v>336</v>
       </c>
@@ -13973,11 +13973,11 @@
       <c r="D140" s="58"/>
       <c r="E140" s="301"/>
       <c r="F140" s="58"/>
-      <c r="G140" s="341" t="s">
+      <c r="G140" s="339" t="s">
         <v>356</v>
       </c>
-      <c r="H140" s="341"/>
-      <c r="I140" s="341"/>
+      <c r="H140" s="339"/>
+      <c r="I140" s="339"/>
       <c r="J140" s="302" t="s">
         <v>357</v>
       </c>
@@ -14408,6 +14408,12 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="C6:E6"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="C11:F11"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="J11:K11"/>
     <mergeCell ref="C96:C110"/>
     <mergeCell ref="C111:C115"/>
     <mergeCell ref="G140:I140"/>
@@ -14418,12 +14424,6 @@
     <mergeCell ref="C36:C41"/>
     <mergeCell ref="C43:C44"/>
     <mergeCell ref="C45:C64"/>
-    <mergeCell ref="C6:E6"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="C11:F11"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="J11:K11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -14473,14 +14473,14 @@
       <c r="D6" s="157"/>
       <c r="E6" s="158"/>
       <c r="F6" s="159"/>
-      <c r="G6" s="361" t="s">
+      <c r="G6" s="367" t="s">
         <v>212</v>
       </c>
-      <c r="H6" s="361"/>
-      <c r="I6" s="361" t="s">
+      <c r="H6" s="367"/>
+      <c r="I6" s="367" t="s">
         <v>213</v>
       </c>
-      <c r="J6" s="361"/>
+      <c r="J6" s="367"/>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="160" t="s">
@@ -14577,14 +14577,14 @@
       <c r="D11" s="169"/>
       <c r="E11" s="169"/>
       <c r="F11" s="105"/>
-      <c r="G11" s="361" t="s">
+      <c r="G11" s="367" t="s">
         <v>212</v>
       </c>
-      <c r="H11" s="361"/>
-      <c r="I11" s="361" t="s">
+      <c r="H11" s="367"/>
+      <c r="I11" s="367" t="s">
         <v>213</v>
       </c>
-      <c r="J11" s="361"/>
+      <c r="J11" s="367"/>
     </row>
     <row r="12" spans="1:10" s="172" customFormat="1" ht="26.45">
       <c r="A12" s="171" t="s">
@@ -15823,12 +15823,12 @@
       </c>
     </row>
     <row r="56" spans="1:8">
-      <c r="A56" s="365" t="s">
+      <c r="A56" s="361" t="s">
         <v>437</v>
       </c>
-      <c r="B56" s="366"/>
-      <c r="C56" s="366"/>
-      <c r="D56" s="367"/>
+      <c r="B56" s="362"/>
+      <c r="C56" s="362"/>
+      <c r="D56" s="363"/>
     </row>
     <row r="57" spans="1:8">
       <c r="A57" s="160" t="s">
@@ -15931,7 +15931,7 @@
       <c r="G64" s="200">
         <v>50</v>
       </c>
-      <c r="H64" s="362">
+      <c r="H64" s="364">
         <v>569250</v>
       </c>
     </row>
@@ -15957,7 +15957,7 @@
       <c r="G65" s="200">
         <v>9</v>
       </c>
-      <c r="H65" s="363"/>
+      <c r="H65" s="365"/>
     </row>
     <row r="66" spans="1:8">
       <c r="A66" s="158"/>
@@ -15971,7 +15971,7 @@
       </c>
       <c r="F66" s="200"/>
       <c r="G66" s="200"/>
-      <c r="H66" s="364"/>
+      <c r="H66" s="366"/>
     </row>
     <row r="67" spans="1:8">
       <c r="A67" s="158"/>
@@ -16005,7 +16005,7 @@
       <c r="G68" s="200">
         <v>1</v>
       </c>
-      <c r="H68" s="362">
+      <c r="H68" s="364">
         <v>1018899.9999999999</v>
       </c>
     </row>
@@ -16031,7 +16031,7 @@
       <c r="G69" s="200">
         <v>1</v>
       </c>
-      <c r="H69" s="363"/>
+      <c r="H69" s="365"/>
     </row>
     <row r="70" spans="1:8">
       <c r="A70" s="158">
@@ -16055,7 +16055,7 @@
       <c r="G70" s="200">
         <v>1</v>
       </c>
-      <c r="H70" s="363"/>
+      <c r="H70" s="365"/>
     </row>
     <row r="71" spans="1:8">
       <c r="A71" s="158">
@@ -16079,7 +16079,7 @@
       <c r="G71" s="200">
         <v>23</v>
       </c>
-      <c r="H71" s="363"/>
+      <c r="H71" s="365"/>
     </row>
     <row r="72" spans="1:8">
       <c r="A72" s="158">
@@ -16103,7 +16103,7 @@
       <c r="G72" s="200">
         <v>17</v>
       </c>
-      <c r="H72" s="363"/>
+      <c r="H72" s="365"/>
     </row>
     <row r="73" spans="1:8">
       <c r="A73" s="158">
@@ -16127,7 +16127,7 @@
       <c r="G73" s="200">
         <v>3</v>
       </c>
-      <c r="H73" s="363"/>
+      <c r="H73" s="365"/>
     </row>
     <row r="74" spans="1:8">
       <c r="A74" s="158">
@@ -16151,7 +16151,7 @@
       <c r="G74" s="200">
         <v>3</v>
       </c>
-      <c r="H74" s="363"/>
+      <c r="H74" s="365"/>
     </row>
     <row r="75" spans="1:8">
       <c r="A75" s="158"/>
@@ -16169,7 +16169,7 @@
       <c r="G75" s="200">
         <v>49</v>
       </c>
-      <c r="H75" s="364"/>
+      <c r="H75" s="366"/>
     </row>
     <row r="76" spans="1:8">
       <c r="A76" s="158"/>
@@ -16203,7 +16203,7 @@
       <c r="G77" s="200">
         <v>3</v>
       </c>
-      <c r="H77" s="362">
+      <c r="H77" s="364">
         <v>1000000</v>
       </c>
     </row>
@@ -16229,7 +16229,7 @@
       <c r="G78" s="200">
         <v>0.5</v>
       </c>
-      <c r="H78" s="363"/>
+      <c r="H78" s="365"/>
     </row>
     <row r="79" spans="1:8">
       <c r="A79" s="158">
@@ -16253,7 +16253,7 @@
       <c r="G79" s="200">
         <v>1</v>
       </c>
-      <c r="H79" s="363"/>
+      <c r="H79" s="365"/>
     </row>
     <row r="80" spans="1:8">
       <c r="A80" s="158">
@@ -16277,7 +16277,7 @@
       <c r="G80" s="200">
         <v>1</v>
       </c>
-      <c r="H80" s="363"/>
+      <c r="H80" s="365"/>
     </row>
     <row r="81" spans="1:8">
       <c r="A81" s="158">
@@ -16301,7 +16301,7 @@
       <c r="G81" s="200">
         <v>10</v>
       </c>
-      <c r="H81" s="363"/>
+      <c r="H81" s="365"/>
     </row>
     <row r="82" spans="1:8">
       <c r="A82" s="158">
@@ -16325,7 +16325,7 @@
       <c r="G82" s="200">
         <v>0.5</v>
       </c>
-      <c r="H82" s="363"/>
+      <c r="H82" s="365"/>
     </row>
     <row r="83" spans="1:8">
       <c r="A83" s="158">
@@ -16349,7 +16349,7 @@
       <c r="G83" s="200">
         <v>0.2</v>
       </c>
-      <c r="H83" s="363"/>
+      <c r="H83" s="365"/>
     </row>
     <row r="84" spans="1:8">
       <c r="A84" s="158">
@@ -16373,7 +16373,7 @@
       <c r="G84" s="200">
         <v>1</v>
       </c>
-      <c r="H84" s="363"/>
+      <c r="H84" s="365"/>
     </row>
     <row r="85" spans="1:8">
       <c r="A85" s="158">
@@ -16397,7 +16397,7 @@
       <c r="G85" s="200">
         <v>1.5</v>
       </c>
-      <c r="H85" s="363"/>
+      <c r="H85" s="365"/>
     </row>
     <row r="86" spans="1:8">
       <c r="A86" s="158">
@@ -16421,7 +16421,7 @@
       <c r="G86" s="200">
         <v>1.5</v>
       </c>
-      <c r="H86" s="364"/>
+      <c r="H86" s="366"/>
     </row>
     <row r="87" spans="1:8">
       <c r="A87" s="158"/>
@@ -16473,7 +16473,7 @@
       <c r="G89" s="200">
         <v>20</v>
       </c>
-      <c r="H89" s="362">
+      <c r="H89" s="364">
         <v>833333</v>
       </c>
     </row>
@@ -16499,7 +16499,7 @@
       <c r="G90" s="200">
         <v>1.5</v>
       </c>
-      <c r="H90" s="363"/>
+      <c r="H90" s="365"/>
     </row>
     <row r="91" spans="1:8">
       <c r="A91" s="158">
@@ -16523,7 +16523,7 @@
       <c r="G91" s="200">
         <v>1.5</v>
       </c>
-      <c r="H91" s="363"/>
+      <c r="H91" s="365"/>
     </row>
     <row r="92" spans="1:8">
       <c r="A92" s="158">
@@ -16547,7 +16547,7 @@
       <c r="G92" s="200">
         <v>0.5</v>
       </c>
-      <c r="H92" s="363"/>
+      <c r="H92" s="365"/>
     </row>
     <row r="93" spans="1:8">
       <c r="A93" s="158">
@@ -16571,7 +16571,7 @@
       <c r="G93" s="200">
         <v>0.5</v>
       </c>
-      <c r="H93" s="363"/>
+      <c r="H93" s="365"/>
     </row>
     <row r="94" spans="1:8">
       <c r="A94" s="158">
@@ -16595,7 +16595,7 @@
       <c r="G94" s="200">
         <v>0.5</v>
       </c>
-      <c r="H94" s="363"/>
+      <c r="H94" s="365"/>
     </row>
     <row r="95" spans="1:8">
       <c r="A95" s="158"/>
@@ -16613,7 +16613,7 @@
       <c r="G95" s="200">
         <v>24.5</v>
       </c>
-      <c r="H95" s="364"/>
+      <c r="H95" s="366"/>
     </row>
     <row r="96" spans="1:8">
       <c r="A96" s="158"/>
@@ -16647,7 +16647,7 @@
       <c r="G97" s="200">
         <v>1</v>
       </c>
-      <c r="H97" s="362">
+      <c r="H97" s="364">
         <v>660000</v>
       </c>
     </row>
@@ -16673,7 +16673,7 @@
       <c r="G98" s="200">
         <v>0.5</v>
       </c>
-      <c r="H98" s="363"/>
+      <c r="H98" s="365"/>
     </row>
     <row r="99" spans="1:8">
       <c r="A99" s="158">
@@ -16697,7 +16697,7 @@
       <c r="G99" s="200">
         <v>1</v>
       </c>
-      <c r="H99" s="363"/>
+      <c r="H99" s="365"/>
     </row>
     <row r="100" spans="1:8">
       <c r="A100" s="158">
@@ -16721,7 +16721,7 @@
       <c r="G100" s="200">
         <v>0.5</v>
       </c>
-      <c r="H100" s="363"/>
+      <c r="H100" s="365"/>
     </row>
     <row r="101" spans="1:8">
       <c r="A101" s="158"/>
@@ -16739,7 +16739,7 @@
       <c r="G101" s="200">
         <v>4</v>
       </c>
-      <c r="H101" s="364"/>
+      <c r="H101" s="366"/>
     </row>
     <row r="102" spans="1:8">
       <c r="A102" s="158"/>
@@ -16773,7 +16773,7 @@
       <c r="G103" s="200">
         <v>3</v>
       </c>
-      <c r="H103" s="362" t="s">
+      <c r="H103" s="364" t="s">
         <v>441</v>
       </c>
     </row>
@@ -16799,7 +16799,7 @@
       <c r="G104" s="200">
         <v>3</v>
       </c>
-      <c r="H104" s="363"/>
+      <c r="H104" s="365"/>
     </row>
     <row r="105" spans="1:8">
       <c r="A105" s="158">
@@ -16823,7 +16823,7 @@
       <c r="G105" s="200">
         <v>1.25</v>
       </c>
-      <c r="H105" s="363"/>
+      <c r="H105" s="365"/>
     </row>
     <row r="106" spans="1:8">
       <c r="A106" s="158">
@@ -16847,7 +16847,7 @@
       <c r="G106" s="200">
         <v>3</v>
       </c>
-      <c r="H106" s="363"/>
+      <c r="H106" s="365"/>
     </row>
     <row r="107" spans="1:8">
       <c r="A107" s="158"/>
@@ -16865,7 +16865,7 @@
       <c r="G107" s="200">
         <v>10.25</v>
       </c>
-      <c r="H107" s="364"/>
+      <c r="H107" s="366"/>
     </row>
     <row r="108" spans="1:8">
       <c r="A108" s="158"/>
@@ -16904,17 +16904,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="H103:H107"/>
     <mergeCell ref="A56:D56"/>
     <mergeCell ref="H68:H75"/>
     <mergeCell ref="H77:H86"/>
     <mergeCell ref="H89:H95"/>
     <mergeCell ref="H97:H101"/>
     <mergeCell ref="H64:H66"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="H103:H107"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -16965,14 +16965,14 @@
       <c r="C6" s="369"/>
       <c r="D6" s="369"/>
       <c r="E6" s="369"/>
-      <c r="F6" s="361" t="s">
+      <c r="F6" s="367" t="s">
         <v>212</v>
       </c>
-      <c r="G6" s="361"/>
-      <c r="H6" s="361" t="s">
+      <c r="G6" s="367"/>
+      <c r="H6" s="367" t="s">
         <v>213</v>
       </c>
-      <c r="I6" s="361"/>
+      <c r="I6" s="367"/>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="52" t="s">
@@ -17060,14 +17060,14 @@
     <row r="11" spans="1:9">
       <c r="A11" s="49"/>
       <c r="B11" s="49"/>
-      <c r="C11" s="361" t="s">
+      <c r="C11" s="367" t="s">
         <v>212</v>
       </c>
-      <c r="D11" s="361"/>
-      <c r="E11" s="361" t="s">
+      <c r="D11" s="367"/>
+      <c r="E11" s="367" t="s">
         <v>213</v>
       </c>
-      <c r="F11" s="361"/>
+      <c r="F11" s="367"/>
     </row>
     <row r="12" spans="1:9" s="71" customFormat="1">
       <c r="A12" s="61" t="s">
@@ -17202,14 +17202,14 @@
       <c r="B19" s="106" t="s">
         <v>215</v>
       </c>
-      <c r="C19" s="361" t="s">
+      <c r="C19" s="367" t="s">
         <v>212</v>
       </c>
-      <c r="D19" s="361"/>
-      <c r="E19" s="361" t="s">
+      <c r="D19" s="367"/>
+      <c r="E19" s="367" t="s">
         <v>213</v>
       </c>
-      <c r="F19" s="361"/>
+      <c r="F19" s="367"/>
     </row>
     <row r="20" spans="1:6" s="71" customFormat="1">
       <c r="A20" s="111"/>
@@ -17752,14 +17752,14 @@
       <c r="C6" s="378"/>
       <c r="D6" s="378"/>
       <c r="E6" s="236"/>
-      <c r="F6" s="361" t="s">
+      <c r="F6" s="367" t="s">
         <v>212</v>
       </c>
-      <c r="G6" s="361"/>
-      <c r="H6" s="361" t="s">
+      <c r="G6" s="367"/>
+      <c r="H6" s="367" t="s">
         <v>213</v>
       </c>
-      <c r="I6" s="361"/>
+      <c r="I6" s="367"/>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="237" t="s">
@@ -17886,14 +17886,14 @@
     <row r="15" spans="1:9" ht="12" customHeight="1">
       <c r="A15" s="240"/>
       <c r="B15" s="236"/>
-      <c r="C15" s="361" t="s">
+      <c r="C15" s="367" t="s">
         <v>212</v>
       </c>
-      <c r="D15" s="361"/>
-      <c r="E15" s="361" t="s">
+      <c r="D15" s="367"/>
+      <c r="E15" s="367" t="s">
         <v>213</v>
       </c>
-      <c r="F15" s="361"/>
+      <c r="F15" s="367"/>
       <c r="G15" s="245"/>
       <c r="H15" s="333" t="s">
         <v>466</v>
@@ -18849,14 +18849,14 @@
       <c r="D8" s="380"/>
       <c r="E8" s="380"/>
       <c r="F8" s="380"/>
-      <c r="G8" s="361" t="s">
+      <c r="G8" s="367" t="s">
         <v>212</v>
       </c>
-      <c r="H8" s="361"/>
-      <c r="I8" s="361" t="s">
+      <c r="H8" s="367"/>
+      <c r="I8" s="367" t="s">
         <v>213</v>
       </c>
-      <c r="J8" s="361"/>
+      <c r="J8" s="367"/>
     </row>
     <row r="9" spans="2:10">
       <c r="B9" s="262" t="s">
@@ -18968,14 +18968,14 @@
     <row r="14" spans="2:10" ht="12" customHeight="1">
       <c r="B14" s="269"/>
       <c r="C14" s="266"/>
-      <c r="D14" s="361" t="s">
+      <c r="D14" s="367" t="s">
         <v>212</v>
       </c>
-      <c r="E14" s="361"/>
-      <c r="F14" s="361" t="s">
+      <c r="E14" s="367"/>
+      <c r="F14" s="367" t="s">
         <v>213</v>
       </c>
-      <c r="G14" s="361"/>
+      <c r="G14" s="367"/>
       <c r="H14" s="315" t="s">
         <v>466</v>
       </c>

</xml_diff>